<commit_message>
feat: agregar historico de avance de obra del proyecto 63 LIVING
Carga los porcentajes de avance mensual (sep-2023 a ago-2025, obra
terminada al 100%) a partir del historico semanal entregado; los
meses posteriores (sep-2025 a jun-2026) se mantienen en 100%.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/InventarioPorProyecto.xlsx
+++ b/public/InventarioPorProyecto.xlsx
@@ -3049,7 +3049,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n"/>
+      <c r="B33" s="5" t="n">
+        <v>0.01</v>
+      </c>
       <c r="C33" s="2" t="n">
         <v>45170</v>
       </c>
@@ -3120,7 +3122,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n"/>
+      <c r="B34" s="5" t="n">
+        <v>0.01</v>
+      </c>
       <c r="C34" s="2" t="n">
         <v>45200</v>
       </c>
@@ -3191,7 +3195,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n"/>
+      <c r="B35" s="5" t="n">
+        <v>0.03</v>
+      </c>
       <c r="C35" s="2" t="n">
         <v>45231</v>
       </c>
@@ -3262,7 +3268,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n"/>
+      <c r="B36" s="5" t="n">
+        <v>0.05</v>
+      </c>
       <c r="C36" s="2" t="n">
         <v>45261</v>
       </c>
@@ -3333,7 +3341,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n"/>
+      <c r="B37" s="5" t="n">
+        <v>0.06</v>
+      </c>
       <c r="C37" s="2" t="n">
         <v>45292</v>
       </c>
@@ -3404,7 +3414,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n"/>
+      <c r="B38" s="5" t="n">
+        <v>0.08</v>
+      </c>
       <c r="C38" s="2" t="n">
         <v>45323</v>
       </c>
@@ -3475,7 +3487,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n"/>
+      <c r="B39" s="5" t="n">
+        <v>0.09</v>
+      </c>
       <c r="C39" s="2" t="n">
         <v>45352</v>
       </c>
@@ -3546,7 +3560,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n"/>
+      <c r="B40" s="5" t="n">
+        <v>0.11</v>
+      </c>
       <c r="C40" s="2" t="n">
         <v>45383</v>
       </c>
@@ -3617,7 +3633,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n"/>
+      <c r="B41" s="5" t="n">
+        <v>0.13</v>
+      </c>
       <c r="C41" s="2" t="n">
         <v>45413</v>
       </c>
@@ -3688,7 +3706,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n"/>
+      <c r="B42" s="5" t="n">
+        <v>0.17</v>
+      </c>
       <c r="C42" s="2" t="n">
         <v>45444</v>
       </c>
@@ -3759,7 +3779,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B43" s="5" t="n"/>
+      <c r="B43" s="5" t="n">
+        <v>0.22</v>
+      </c>
       <c r="C43" s="2" t="n">
         <v>45474</v>
       </c>
@@ -3830,7 +3852,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B44" s="5" t="n"/>
+      <c r="B44" s="5" t="n">
+        <v>0.24</v>
+      </c>
       <c r="C44" s="2" t="n">
         <v>45505</v>
       </c>
@@ -3901,7 +3925,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B45" s="5" t="n"/>
+      <c r="B45" s="5" t="n">
+        <v>0.29</v>
+      </c>
       <c r="C45" s="2" t="n">
         <v>45536</v>
       </c>
@@ -3972,7 +3998,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n"/>
+      <c r="B46" s="5" t="n">
+        <v>0.37</v>
+      </c>
       <c r="C46" s="2" t="n">
         <v>45566</v>
       </c>
@@ -4043,7 +4071,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n"/>
+      <c r="B47" s="5" t="n">
+        <v>0.46</v>
+      </c>
       <c r="C47" s="2" t="n">
         <v>45597</v>
       </c>
@@ -4114,7 +4144,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n"/>
+      <c r="B48" s="5" t="n">
+        <v>0.62</v>
+      </c>
       <c r="C48" s="2" t="n">
         <v>45627</v>
       </c>
@@ -4185,7 +4217,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n"/>
+      <c r="B49" s="5" t="n">
+        <v>0.6899999999999999</v>
+      </c>
       <c r="C49" s="2" t="n">
         <v>45658</v>
       </c>
@@ -4256,7 +4290,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n"/>
+      <c r="B50" s="5" t="n">
+        <v>0.78</v>
+      </c>
       <c r="C50" s="2" t="n">
         <v>45689</v>
       </c>
@@ -4327,7 +4363,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n"/>
+      <c r="B51" s="5" t="n">
+        <v>0.82</v>
+      </c>
       <c r="C51" s="2" t="n">
         <v>45717</v>
       </c>
@@ -4398,7 +4436,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B52" s="5" t="n"/>
+      <c r="B52" s="5" t="n">
+        <v>0.87</v>
+      </c>
       <c r="C52" s="2" t="n">
         <v>45748</v>
       </c>
@@ -4469,7 +4509,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n"/>
+      <c r="B53" s="5" t="n">
+        <v>0.91</v>
+      </c>
       <c r="C53" s="2" t="n">
         <v>45778</v>
       </c>
@@ -4540,7 +4582,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B54" s="5" t="n"/>
+      <c r="B54" s="5" t="n">
+        <v>0.95</v>
+      </c>
       <c r="C54" s="2" t="n">
         <v>45809</v>
       </c>
@@ -4611,7 +4655,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n"/>
+      <c r="B55" s="5" t="n">
+        <v>0.99</v>
+      </c>
       <c r="C55" s="2" t="n">
         <v>45839</v>
       </c>
@@ -4682,7 +4728,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n"/>
+      <c r="B56" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C56" s="2" t="n">
         <v>45870</v>
       </c>
@@ -4753,7 +4801,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B57" s="5" t="n"/>
+      <c r="B57" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C57" s="2" t="n">
         <v>45901</v>
       </c>
@@ -4824,7 +4874,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n"/>
+      <c r="B58" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C58" s="2" t="n">
         <v>45931</v>
       </c>
@@ -4895,7 +4947,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n"/>
+      <c r="B59" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C59" s="2" t="n">
         <v>45962</v>
       </c>
@@ -4966,7 +5020,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B60" s="5" t="n"/>
+      <c r="B60" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C60" s="2" t="n">
         <v>45992</v>
       </c>
@@ -5037,7 +5093,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B61" s="5" t="n"/>
+      <c r="B61" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C61" s="2" t="n">
         <v>46023</v>
       </c>
@@ -5108,7 +5166,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B62" s="5" t="n"/>
+      <c r="B62" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C62" s="2" t="n">
         <v>46054</v>
       </c>
@@ -5179,7 +5239,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B63" s="5" t="n"/>
+      <c r="B63" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C63" s="2" t="n">
         <v>46082</v>
       </c>
@@ -5250,7 +5312,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n"/>
+      <c r="B64" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C64" s="2" t="n">
         <v>46113</v>
       </c>
@@ -5321,7 +5385,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B65" s="5" t="n"/>
+      <c r="B65" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C65" s="2" t="n">
         <v>46143</v>
       </c>
@@ -5392,7 +5458,9 @@
           <t>63 LIVING</t>
         </is>
       </c>
-      <c r="B66" s="5" t="n"/>
+      <c r="B66" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="C66" s="2" t="n">
         <v>46174</v>
       </c>

</xml_diff>